<commit_message>
data: update HWV, RV, composers
</commit_message>
<xml_diff>
--- a/xlsx/HWV.xlsx
+++ b/xlsx/HWV.xlsx
@@ -2470,7 +2470,7 @@
     <t>Motet</t>
   </si>
   <si>
-    <t>motet pour soprano avec cordes (2 violons) et basse continue</t>
+    <t>soprano avec cordes (2 violons) et basse continue</t>
   </si>
   <si>
     <t>pour la fête de St. Antoine de Padoue
@@ -2569,7 +2569,7 @@
     <t>O qualis de coelo sonus</t>
   </si>
   <si>
-    <t>motet pour soprano solo avec cordes (2 violons) et basse continue</t>
+    <t>soprano solo avec cordes (2 violons) et basse continue</t>
   </si>
   <si>
     <t>HWV 240</t>
@@ -2578,7 +2578,7 @@
     <t>Saeviat tellus inter rigores</t>
   </si>
   <si>
-    <t>motet pour soprano solo avec orchestre (2 hautbois, 2 violons, alto) et basse continue</t>
+    <t>soprano solo avec orchestre (2 hautbois, 2 violons, alto) et basse continue</t>
   </si>
   <si>
     <t>pour la Madonne très sainte de Carmine
@@ -2603,7 +2603,7 @@
     <t>Silete venti</t>
   </si>
   <si>
-    <t>motet pour soprano solo avec orrchestre (2 hautbois, basson, 2 violons, alto, violoncelle) et basse continue</t>
+    <t>soprano solo avec orrchestre (2 hautbois, basson, 2 violons, alto, violoncelle) et basse continue</t>
   </si>
   <si>
     <t>HWV 243</t>
@@ -2624,7 +2624,7 @@
     <t>Kyrie eleison</t>
   </si>
   <si>
-    <t>pour 4 voix (SATB) avec cordes (2 violons, 2 altos) et basse continue</t>
+    <t>4 voix (SATB) avec cordes (2 violons, 2 altos) et basse continue</t>
   </si>
   <si>
     <t>HWV 245</t>
@@ -2633,7 +2633,7 @@
     <t>Gloria in excelsis Deo</t>
   </si>
   <si>
-    <t>pour 5-6 voix (SSATTB) avec orchestre (hautbois, trompette, 2 violons, 2 altos), orgue et basse continue</t>
+    <t>5-6 voix (SSATTB) avec orchestre (hautbois, trompette, 2 violons, 2 altos), orgue et basse continue</t>
   </si>
   <si>
     <t>HWV 269</t>
@@ -7490,13 +7490,10 @@
     <col min="4" max="4" width="26.7117117117117" style="1" customWidth="1"/>
     <col min="5" max="5" width="16.9099099099099" style="2" customWidth="1"/>
     <col min="6" max="6" width="13.5855855855856" style="2" customWidth="1"/>
-    <col min="7" max="7" width="22.1621621621622" style="1" customWidth="1"/>
+    <col min="7" max="7" width="42.9369369369369" style="1" customWidth="1"/>
     <col min="8" max="8" width="36.8378378378378" style="1" customWidth="1"/>
     <col min="9" max="9" width="48.8828828828829" style="1" customWidth="1"/>
-    <col min="10" max="10" width="8.61261261261261" style="1"/>
-    <col min="11" max="11" width="19.4594594594595" style="1" customWidth="1"/>
-    <col min="12" max="16381" width="8.61261261261261" style="1"/>
-    <col min="16383" max="16384" width="8.61261261261261" style="1"/>
+    <col min="10" max="16384" width="8.61261261261261" style="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="16.7" spans="1:9">
@@ -21674,7 +21671,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="C1:E1 G1 I1" formula="1"/>
+    <ignoredError sqref="I1 G1 C1:E1" formula="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>